<commit_message>
Add People Risk tab with shortlist for direct conversations
Adds a new tab (positioned right after Feedback Responses) capturing the
12 people flagged from the written feedback and the engineering 1-5
competency tables: distress/disengagement signals, one conduct issue
routed to HR rather than a chat, an engineering performance-coaching
case, a career-pathway conversation, and two retention risks among
strong performers. Each row carries the category, source page, the
evidence quote, why it was flagged, a suggested next step, and a blank
Status/notes column for tracking outcomes as conversations happen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181H7bukYjEb3tTsSEDdFCz
</commit_message>
<xml_diff>
--- a/Employee_Feedback_Consolidated_2026.xlsx
+++ b/Employee_Feedback_Consolidated_2026.xlsx
@@ -8,12 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feedback Responses" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="People Risk" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chart Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feedback Responses'!$A$1:$P$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'People Risk'!$A$5:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -22,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,17 +43,37 @@
       <sz val="16"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="0055606B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="008E44AD"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="002E6F9E"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F8A70"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00B7791F"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="001F3B57"/>
       <sz val="12"/>
     </font>
     <font>
       <b val="1"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="0055606B"/>
-      <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
@@ -103,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,12 +137,33 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -9719,6 +9762,547 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>People Risk — shortlist for direct conversations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Not an exhaustive scan — a curated read of tone and word choice in the written answers, plus the engineering 1-5 ratings. Treat as a starting point to sanity-check against what you already know of each person, not a verdict. Fill in Status/Notes as conversations happen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5" ht="32" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B5" s="1" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C5" s="1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="E5" s="1" t="inlineStr">
+        <is>
+          <t>What they said / the evidence</t>
+        </is>
+      </c>
+      <c r="F5" s="1" t="inlineStr">
+        <is>
+          <t>Why it's flagged</t>
+        </is>
+      </c>
+      <c r="G5" s="1" t="inlineStr">
+        <is>
+          <t>Suggested next step</t>
+        </is>
+      </c>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>Status / notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Mitchell Frick</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Engineering docx, Mitchell Frick section</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Self-rated himself well below his manager across the 1-5 competency tables (self average 2.56/5 vs manager 3.44/5, a -0.88 gap — the only person in the cohort to self-rate below their manager by this much).</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>A sharp negative self-vs-manager gap like this usually means low confidence, a rough stretch, or being harder on himself than the situation warrants — worth a direct, supportive conversation rather than reading it off the form.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Quiet one-on-one check-in, not a performance conversation.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>John Visintin ("John V.")</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Forms 3, p35-36</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>52 years' experience, 3 months from his 70th birthday. Asked for a 4-day/32hr week in December and was refused. Wrote: "I think there lies a lack of compassion."</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>The most fixable item on this list — a specific, denied request from someone with enormous tenure, not a vague morale problem.</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Revisit the request itself, not just the conversation.</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8" ht="60" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ghayas Ul Haq ("Haq")</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Forms 3, p59-60</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Rated the past year "Bad" — "I will say the worst because of the workload and processes." Says the role "does not suit and fulfil what my career aspirations were" (noted as a temp).</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Telling you plainly, in writing, that he isn't staying.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Direct conversation about what would change the trajectory, if anything.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="60" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Chaudhary Saqib</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Forms 3, p65-66</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>"Bad ... overloaded with work with under payment/reward." No WFH days, pay "under payment compared to market." Temp; not on the personnel register.</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Same profile as Haq — overloaded, underpaid, and says so directly.</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Check whether pay/workload for this role is out of line with market.</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10" ht="60" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Jurgen Cassar</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Forms 1, p21-22</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>"Constantly told we are failing - always feeling defeated + no feedback or guidance to improve." Least-liked part of the job: "Constant feel of defeat."</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Reads like someone being worn down by criticism with no support attached to it.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Check in on how feedback is currently being delivered to him.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Likely Kalim Broom (unconfirmed — illegible signature)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Forms 2, p47-48</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Ticked "I'm not doing the work I was employed for." Wrote about being handed jobs he isn't qualified for with no support to finish them "in a timely and proficient manner."</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Strong disengagement signal. Name is a plausible-but-unconfirmed guess by elimination against the personnel register — confirm who this is before acting.</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>Confirm identity with the floor supervisor first, then check in.</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="60" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Distress / disengagement</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Luong Ha</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Forms 3, p9-10</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ticked "haven't enjoyed doing the work I was employed for" and "can do but doesn't interest me." Called it an "unsafe working environment."</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Disengagement plus a safety complaint — the safety part needs looking at regardless of the morale question.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Follow up on the specific safety concern; separately, check in on role fit.</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="60" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Conduct — needs HR, not just a chat</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Likely Bhupinder Singh ("A BS")</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Forms 2, p9-10</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Raised "lots of misogyny / some racism," and wrote that some supervisors "use their yellow shirt to abuse their power," plus lunchroom gossip about staff by other supervisors.</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>A conduct allegation, not a morale dip — different in kind from everything else here.</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>Route to HR rather than handling as a one-on-one check-in.</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="60" customHeight="1">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Performance coaching (engineering ratings)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Liam McNamara</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Engineering docx, Liam McNamara section</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Lowest average in the engineering cohort (2.68/5 manager rating), specifically Organisation and Attendance &amp; Punctuality both at 2/5. His self-ratings ran higher than his manager's almost everywhere (+0.56 gap).</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>A different pattern to Mitchell Frick — looks more like a blind spot than unhappiness, since he rates himself higher than his manager does.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Direct, constructive conversation about the specific gap areas.</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="60" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>Career pathway conversation</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Luke Moran</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Engineering docx, Luke Moran section</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Self-rated slightly below his manager (-0.18 gap). Annotated "More looking into an engineering position" next to the (unticked) "This is my chosen career path" box.</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Sounds like someone who wants a different lane, not someone who wants out.</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>Conversation about a path toward the engineering role he's signalling interest in.</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="60" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Retention risk — strong performer</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Sai Vivek Yedlapati</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Engineering docx, Sai Vivek Yedlapati section</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Highest-rated engineer in the cohort (4.35/5 average, zero gap between self and manager ratings). Wrote explicitly: "I need to see growth for long term development (like management level)."</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Top performers who say this out loud and see nothing change are exactly the ones who leave quietly.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Proactive conversation about a growth/leadership pathway, before he goes looking elsewhere.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Retention risk — strong performer</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Josh Kalms ("Josh K")</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Workshop</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Forms 3, p63-64</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Manager notes already on the form (initialled "TB") say he's unsure about staying long-term and feels leadership under-delivers.</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>This one was already flagged once, by a manager, on the form itself.</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>Check whether anything came of the earlier notes; follow up if not.</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:H17"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9734,19 +10318,19 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>Q1 — How would you rate your working experience at Liquip Victoria?</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="14" t="inlineStr">
         <is>
           <t>Response option</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>Number of people</t>
         </is>
@@ -9853,19 +10437,19 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>Q1.1 — Has the past year been good / satisfactory / bad for you?</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Response option</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Number of people</t>
         </is>
@@ -9912,19 +10496,19 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="13" t="inlineStr">
         <is>
           <t>Q2 — How would you rate working for this organisation?</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="6" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Response option</t>
         </is>
       </c>
-      <c r="B26" s="6" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>Number of people</t>
         </is>
@@ -10021,19 +10605,19 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>Q5 — How would you rate your interest in this role?</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="6" t="inlineStr">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>Response option</t>
         </is>
       </c>
-      <c r="B39" s="6" t="inlineStr">
+      <c r="B39" s="14" t="inlineStr">
         <is>
           <t>Number of people</t>
         </is>
@@ -10134,7 +10718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10154,7 +10738,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Multiple-choice questions are shown as bar / pie charts. Written answers are shown as word clouds: green = positive inference, red = negative inference, grey = used about equally either way. Word size = how often the word appears across all responses.</t>
         </is>
@@ -10171,7 +10755,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10192,144 +10776,144 @@
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Three scanned bundles (Employee Feedback forms 1, 2 and 3 — 40, 94 and 68 pages) covering the 87 workshop/office respondents, plus 11 engineering team reviews supplied separately: eight as sections of one Word document and three as individually typed PDFs (Josh Cho, Muhammad Saad Zia, Patrick Tio). Every page was read individually.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Coverage</t>
         </is>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>98 completed feedback forms are recorded, one row each, on the 'Feedback Responses' tab — 87 workshop/office plus 11 engineering, distinguished by the Team column.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Blank pages</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>The three scanned bundles were duplex-scanned, so sheets printed single-sided produced blank backs. Blank pages were skipped and the following page was used, so no respondent was lost. Blank backs found: Forms 1 p6; Forms 2 p73, 78, 85, 88, 90; Forms 3 p20, 22, 24, 26, 28, 30, 54, 56, 68.</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Questions captured</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Q1, Q1.1, Q2, Q2.1 (likes and dislikes split into two columns), Q3, Q4, Q5 and Q5.1 (most and least split into two columns). Q6 (core values) was excluded as requested.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Longer forms</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Nine workshop/office people (Hayden, Stanton Thompson, Paul Cini, Ondrej Vujtek, Braden Anderson, Christian Cubrig, James Morris, Alison Chetcuti, Chaudhary Saqib) and all eleven engineering reviews used a typed 13/14/15-page layout, where the same questions run across two or three pages. Those pages were merged into one row per person.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Forms left largely unanswered</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Three workshop people ticked boxes but left the written questions blank or nearly blank: Alex (Forms 2, p43–44 — only Q1, Q2 and Q5 ticks plus 'Quality' at Q6); Pat (Forms 3, p7–8 — all ticks completed, every written answer blank); Greg (Forms 3, p37–38 — Q2.1 answered, then Q3, Q4, Q5 and Q5.1 all blank).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Engineering checkbox limits</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>Two engineering sections (Ehsan Barani and Vahid Shirazi) use an older Word form-field format for their tick-boxes that could not be read reliably from the document's XML, so Q1/Q1.1/Q2/Q5 are marked 'Not extractable' rather than guessed — their written answers are transcribed in full and are not affected.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="75" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Names not legible</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>Nine forms carry a name that isn't fully legible or fully certain: one signed with initials read as 'JW', one 'A BS', one 'BA', two illegible signatures, one cover with no name at all (a safety role), and three more ('Gavin', 'Steve', 'Joseph') where the register has two or more people the handwriting could equally be. Column D records what can be inferred, cross-checked against the personnel register.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="75" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Personnel register</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>The personnel register (137 names) was supplied and used to check every name on the 'Feedback Responses' tab — see column D. Most first-name-only or misspelled entries were resolved to a single register entry; a handful remain genuinely ambiguous (two people with the same first name and no other clue) or unresolved (no register entry fits), and those are flagged as such in column D rather than guessed.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="90" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Engineering team reviews</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>All eleven requested engineering reviews are now included: Abin Eldos, Behzad Moazeni, Ehsan Barani, Liam McNamara, Luke Moran, Mitchell Frick, Sai Vivek Yedlapati and Vahid Shirazi came as sections of one Word document (eng_master_word); Josh Cho, Muhammad Saad Zia and Patrick Tio came as individually typed PDFs. Each engineering review used the same feedback questions as the workshop form, laid out across a 13–14 page typed template that also carries a separate job-performance/KPI section (not requested and not included here).</t>
         </is>
       </c>
     </row>
     <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Word cloud colours</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Green = the word appears in positive contexts (Q2.1 likes, Q5.1 'most'); red = negative contexts (Q2.1 dislikes, Q5.1 'least', Q3 change requests, Q4 difficulties); grey = the word is used about equally both ways. Shade intensity follows how one-sided the usage is.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Transcription</t>
         </is>
       </c>
-      <c r="B14" s="9" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>Handwriting was transcribed as faithfully as possible; obvious spelling slips were kept, and uncertain readings are flagged in the Notes column or with a question mark.</t>
         </is>

</xml_diff>

<commit_message>
Add Rita Kelly's feedback form (99th response)
Single standalone scanned page (the typed 'Employee's Feedback' page,
2 of 13) with no cover page or signature — name confirmed by Geoff and
matched to the personnel register (Kelly, Rita), which was previously
unmatched to any other form. Ruled out as a candidate for the still-
unresolved unnamed safety-role form, since she now has her own
confirmed submission. Charts and word clouds updated to include her.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0181H7bukYjEb3tTsSEDdFCz
</commit_message>
<xml_diff>
--- a/Employee_Feedback_Consolidated_2026.xlsx
+++ b/Employee_Feedback_Consolidated_2026.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feedback Responses'!$A$1:$P$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Feedback Responses'!$A$1:$P$100</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'People Risk'!$A$5:$H$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1085,7 +1085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P99"/>
+  <dimension ref="A1:P100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8534,7 +8534,7 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>Unresolved — safety/HSE role; possible register candidates not otherwise matched in this set include Rita Kelly, Tanja Koch and Lara Greene, but nothing in the form ties it to any one of them</t>
+          <t>Unresolved — safety/HSE role; possible register candidates not otherwise matched in this set include Tanja Koch and Lara Greene (Rita Kelly is now ruled out — she has her own separate, confirmed submission), but nothing in the form ties it to either remaining candidate</t>
         </is>
       </c>
       <c r="E86" s="2" t="inlineStr">
@@ -8773,22 +8773,22 @@
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Workshop</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>Abin Eldos</t>
+          <t>Rita Kelly</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>Confirmed — exact match (register: Eldos, Abin)</t>
+          <t>Confirmed by Geoff — exact match (register: Kelly, Rita); previously unmatched to any other form in the set</t>
         </is>
       </c>
       <c r="E89" s="3" t="inlineStr">
         <is>
-          <t>Engineering docx, Abin Eldos section</t>
+          <t>Standalone scan, single page (no cover/signature)</t>
         </is>
       </c>
       <c r="F89" s="3" t="inlineStr">
@@ -8807,357 +8807,6 @@
         </is>
       </c>
       <c r="H89" s="3" t="inlineStr">
-        <is>
-          <t>• Good culture within organisation
-• Helpful / approachable supervisors
-• Career development opportunities
-• There is a good team of employees
-• There is opportunity to grow within the company
-• Recommend this company to others</t>
-        </is>
-      </c>
-      <c r="I89" s="3" t="inlineStr">
-        <is>
-          <t>Supportive and friendly team environment, opportunities to learn new skills/experience, approachable team</t>
-        </is>
-      </c>
-      <c r="J89" s="3" t="inlineStr">
-        <is>
-          <t>Communication between team could be improved, less work-life balance</t>
-        </is>
-      </c>
-      <c r="K89" s="3" t="inlineStr">
-        <is>
-          <t>Offering additional training and professional development opportunities. Employee Assistance programs</t>
-        </is>
-      </c>
-      <c r="L89" s="3" t="inlineStr">
-        <is>
-          <t>Managing priorities during a busy period with limited timeframe</t>
-        </is>
-      </c>
-      <c r="M89" s="3" t="inlineStr">
-        <is>
-          <t>• I enjoy working in this role
-• I want to stay in this area of work
-• This role fulfils my needs and expectations</t>
-        </is>
-      </c>
-      <c r="N89" s="3" t="inlineStr">
-        <is>
-          <t>Working with diverse range of people and seeing the impact on my work. Electrical design aspects</t>
-        </is>
-      </c>
-      <c r="O89" s="3" t="inlineStr">
-        <is>
-          <t>Routine administrative tasks</t>
-        </is>
-      </c>
-      <c r="P89" s="3" t="inlineStr">
-        <is>
-          <t>Engineering team; supplied separately as a typed docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="96" customHeight="1">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C90" s="2" t="inlineStr">
-        <is>
-          <t>Behzad Moazeni</t>
-        </is>
-      </c>
-      <c r="D90" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed — exact match (register: Moazeni, Behzad)</t>
-        </is>
-      </c>
-      <c r="E90" s="2" t="inlineStr">
-        <is>
-          <t>Engineering docx, Behzad Moazeni section</t>
-        </is>
-      </c>
-      <c r="F90" s="2" t="inlineStr">
-        <is>
-          <t>• I like the team that I work with
-• I have learnt a lot of new things
-• I get along really well with my supervisor
-• I have enjoyed doing the work I was employed for
-• Other: Learnt a bit about pneumatic and fuelling logic</t>
-        </is>
-      </c>
-      <c r="G90" s="2" t="inlineStr">
-        <is>
-          <t>Satisfactory</t>
-        </is>
-      </c>
-      <c r="H90" s="2" t="inlineStr">
-        <is>
-          <t>• Helpful / approachable supervisors
-• There is a good team of employees</t>
-        </is>
-      </c>
-      <c r="I90" s="2" t="inlineStr">
-        <is>
-          <t>Supportive and agreeable colleagues and supervisor. Relative freedom while working on new project (R&amp;D type and SBT/depots). PLC Programming, specially structured text Programming. Rare cases of fault findings</t>
-        </is>
-      </c>
-      <c r="J90" s="2" t="inlineStr">
-        <is>
-          <t>Car park situation (same as last year). Printer too close to the desk. Work planning and prioritization - priorities change multiple times, resulting in mistakes while hopping between tasks; high-priority work is sometimes taken off schedule for months. Lack of clear project specification and expectations at the start of engineering work, and ever-changing specifications. Lack of a clear single stakeholder per project. Untimely project sales handover. Crowded, noisy office space with no dedicated meeting room. Part suppliers' restrictions. Unclear time gap between design and manufacturing. Widespread mindset that Engineering is always responsible for issues. Forced shut-downs using about 40% of paid annual leave without consultation. Not being included in some email chains/discussions but expected to know everything</t>
-        </is>
-      </c>
-      <c r="K90" s="2" t="inlineStr">
-        <is>
-          <t>A clear understanding of the financial aspects of projects' contracts would support better decision-making during the design phase, especially for non-aviation projects. Investment in employees' training and delivering on past promises. Considering Engineering as a finite resource rather than unlimited overhead. Investment in purpose-built tools (i.e. software)</t>
-        </is>
-      </c>
-      <c r="L90" s="2" t="inlineStr">
-        <is>
-          <t>Dealing with other departments. Company having different standards and expectations for different individuals</t>
-        </is>
-      </c>
-      <c r="M90" s="2" t="inlineStr">
-        <is>
-          <t>• This is my chosen career path
-• I enjoy working in this role
-• I want to stay in this area of work
-• This role fulfils my needs and expectations
-• Other: I enjoy the role, but to be honest, I'm not sure about my future</t>
-        </is>
-      </c>
-      <c r="N90" s="2" t="inlineStr">
-        <is>
-          <t>Going over new designs, control logics, and R&amp;D type projects, investigating new products/standards, and trying to analyse systems and/or fault find. Also enjoyed programming while setting up the CAN interface on Volvo FMs</t>
-        </is>
-      </c>
-      <c r="O90" s="2" t="inlineStr">
-        <is>
-          <t>Copy &amp; pasting with minor changes and having to do unnecessary reworks due to last-minute spec changes</t>
-        </is>
-      </c>
-      <c r="P90" s="2" t="inlineStr">
-        <is>
-          <t>Engineering team; supplied separately as a typed docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="96" customHeight="1">
-      <c r="A91" s="3" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C91" s="3" t="inlineStr">
-        <is>
-          <t>Ehsan Barani</t>
-        </is>
-      </c>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed by elimination — the register entry Barani, Ehsan is the only name from the requested engineering list not otherwise accounted for in this document, matching this unnamed section</t>
-        </is>
-      </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>Engineering docx, unnamed section between Behzad Moazeni and Liam McNamara</t>
-        </is>
-      </c>
-      <c r="F91" s="3" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="G91" s="3" t="inlineStr">
-        <is>
-          <t>Not extractable (older form-field format)</t>
-        </is>
-      </c>
-      <c r="H91" s="3" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="I91" s="3" t="inlineStr">
-        <is>
-          <t>I enjoy working in a challenging environment that encourages continuous learning and professional growth. Since joining the company, I have gained valuable new skills and experience through solving complex technical problems. I also appreciate the supportive engineering team, where colleagues are willing to share knowledge and help one another. I enjoy the work I was employed to do and see opportunities to continue developing my career with the company</t>
-        </is>
-      </c>
-      <c r="J91" s="3" t="inlineStr">
-        <is>
-          <t>Car park</t>
-        </is>
-      </c>
-      <c r="K91" s="3" t="inlineStr">
-        <is>
-          <t>Providing additional training opportunities and dedicated time for professional development in key technical areas would help employees continue building their skills and knowledge. Improving the availability of parking spaces for the engineering team would also enhance convenience and the overall workplace experience</t>
-        </is>
-      </c>
-      <c r="L91" s="3" t="inlineStr">
-        <is>
-          <t>I find it most challenging when working on new and unfamiliar tasks under tight deadlines. Balancing rapid learning with delivering accurate, high-quality work can be demanding, but I enjoy the challenge and the opportunity to grow</t>
-        </is>
-      </c>
-      <c r="M91" s="3" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="N91" s="3" t="inlineStr">
-        <is>
-          <t>I am most interested in the variety of engineering work and the opportunity to continuously learn new skills. I have particularly enjoyed gaining experience in hydraulic and pneumatic systems, which were new areas for me</t>
-        </is>
-      </c>
-      <c r="O91" s="3" t="inlineStr">
-        <is>
-          <t>There are no significant aspects of my role that I find least interesting, as each task offers valuable learning opportunities</t>
-        </is>
-      </c>
-      <c r="P91" s="3" t="inlineStr">
-        <is>
-          <t>Name not given on this form; identified by elimination as the remaining name on the engineering list (Ehsan Barani), positioned between Behzad Moazeni and Liam McNamara in the document. This section's tick-boxes use an older Word form-field format that could not be read reliably, so Q1/Q1.1/Q2/Q5 are left blank rather than guessed; the written answers are transcribed in full.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="96" customHeight="1">
-      <c r="A92" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C92" s="2" t="inlineStr">
-        <is>
-          <t>Liam McNamara</t>
-        </is>
-      </c>
-      <c r="D92" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed — exact match (register: McNamara, Liam)</t>
-        </is>
-      </c>
-      <c r="E92" s="2" t="inlineStr">
-        <is>
-          <t>Engineering docx, Liam McNamara section</t>
-        </is>
-      </c>
-      <c r="F92" s="2" t="inlineStr">
-        <is>
-          <t>• I like the team that I work with
-• I have learnt a lot of new things
-• The job is what I expected it to be
-• I get along really well with my supervisor
-• I have enjoyed doing the work I was employed for
-• I see myself developing further with this company</t>
-        </is>
-      </c>
-      <c r="G92" s="2" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="H92" s="2" t="inlineStr">
-        <is>
-          <t>• Good culture within organisation
-• Helpful / approachable supervisors
-• Recommend this company to others
-• There is a good team of employees
-• Practices to encourage social / employee involvement</t>
-        </is>
-      </c>
-      <c r="I92" s="2" t="inlineStr">
-        <is>
-          <t>Good team, good company culture. Reasonable expectations regarding initial domain specific knowledge</t>
-        </is>
-      </c>
-      <c r="J92" s="2" t="inlineStr">
-        <is>
-          <t>Pressuring other departments with a visibly heavier workload than my own to finish jobs</t>
-        </is>
-      </c>
-      <c r="K92" s="2" t="inlineStr">
-        <is>
-          <t>Improve time sheet / job logging system. Separate break and meeting rooms. More parking</t>
-        </is>
-      </c>
-      <c r="L92" s="2" t="inlineStr">
-        <is>
-          <t>Coordinating warranty with other departments. Settling large sets of fleetwide warranty claims</t>
-        </is>
-      </c>
-      <c r="M92" s="2" t="inlineStr">
-        <is>
-          <t>• I enjoy working in this role
-• This role fulfils my needs and expectations</t>
-        </is>
-      </c>
-      <c r="N92" s="2" t="inlineStr">
-        <is>
-          <t>Trialling new design features and R&amp;D work, such as the 360 degree camera setup</t>
-        </is>
-      </c>
-      <c r="O92" s="2" t="inlineStr">
-        <is>
-          <t>Troubleshooting web development issues on the ATG portal</t>
-        </is>
-      </c>
-      <c r="P92" s="2" t="inlineStr">
-        <is>
-          <t>Engineering team; supplied separately as a typed docx</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="96" customHeight="1">
-      <c r="A93" s="3" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="3" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C93" s="3" t="inlineStr">
-        <is>
-          <t>Luke Moran</t>
-        </is>
-      </c>
-      <c r="D93" s="3" t="inlineStr">
-        <is>
-          <t>Confirmed — exact match (register: Moran, Luke)</t>
-        </is>
-      </c>
-      <c r="E93" s="3" t="inlineStr">
-        <is>
-          <t>Engineering docx, Luke Moran section</t>
-        </is>
-      </c>
-      <c r="F93" s="3" t="inlineStr">
-        <is>
-          <t>• I like the team that I work with
-• I have learnt a lot of new things
-• The job is what I expected it to be
-• I get along really well with my supervisor
-• I have enjoyed doing the work I was employed for
-• I see myself developing further with this company</t>
-        </is>
-      </c>
-      <c r="G93" s="3" t="inlineStr">
-        <is>
-          <t>Good</t>
-        </is>
-      </c>
-      <c r="H93" s="3" t="inlineStr">
         <is>
           <t>• Good communication within organisation
 • Helpful / approachable supervisors
@@ -9169,45 +8818,398 @@
 • Practices to encourage social / employee involvement</t>
         </is>
       </c>
+      <c r="I89" s="3" t="inlineStr">
+        <is>
+          <t>Love the growth</t>
+        </is>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>Dislike the different levels of authorities eg: spending verses approvals</t>
+        </is>
+      </c>
+      <c r="K89" s="3" t="inlineStr">
+        <is>
+          <t>Trim the over resourced departments may reduce the errors</t>
+        </is>
+      </c>
+      <c r="L89" s="3" t="inlineStr">
+        <is>
+          <t>Fearing surprises</t>
+        </is>
+      </c>
+      <c r="M89" s="3" t="inlineStr">
+        <is>
+          <t>• This is my chosen career path
+• I enjoy working in this role
+• I want to stay in this area of work
+• This role fulfils my needs and expectations</t>
+        </is>
+      </c>
+      <c r="N89" s="3" t="inlineStr">
+        <is>
+          <t>Teaching others eg: RTR</t>
+        </is>
+      </c>
+      <c r="O89" s="3" t="inlineStr">
+        <is>
+          <t>Under estimated</t>
+        </is>
+      </c>
+      <c r="P89" s="3" t="inlineStr">
+        <is>
+          <t>Provided separately as a single scanned page (page 2 of 13, the typed 'Employee's Feedback' page) with no cover page or signature. Name confirmed by Geoff as Rita Kelly, matching the personnel register (Kelly, Rita) which was previously unmatched to any other form. Annotated 'Continue to build the team for the future' against Q1 Other (box not ticked) and 'Ongoing learning to strengthen Team' against Q1.1 Other (box not ticked). Q6 (core values) answered but excluded per usual scope.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="96" customHeight="1">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Abin Eldos</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed — exact match (register: Eldos, Abin)</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Engineering docx, Abin Eldos section</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>• I like the team that I work with
+• I have learnt a lot of new things
+• The job is what I expected it to be
+• I get along really well with my supervisor
+• I have enjoyed doing the work I was employed for
+• I see myself developing further with this company</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>• Good culture within organisation
+• Helpful / approachable supervisors
+• Career development opportunities
+• There is a good team of employees
+• There is opportunity to grow within the company
+• Recommend this company to others</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
+        <is>
+          <t>Supportive and friendly team environment, opportunities to learn new skills/experience, approachable team</t>
+        </is>
+      </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>Communication between team could be improved, less work-life balance</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>Offering additional training and professional development opportunities. Employee Assistance programs</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>Managing priorities during a busy period with limited timeframe</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>• I enjoy working in this role
+• I want to stay in this area of work
+• This role fulfils my needs and expectations</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Working with diverse range of people and seeing the impact on my work. Electrical design aspects</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>Routine administrative tasks</t>
+        </is>
+      </c>
+      <c r="P90" s="2" t="inlineStr">
+        <is>
+          <t>Engineering team; supplied separately as a typed docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="96" customHeight="1">
+      <c r="A91" s="3" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>Behzad Moazeni</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed — exact match (register: Moazeni, Behzad)</t>
+        </is>
+      </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>Engineering docx, Behzad Moazeni section</t>
+        </is>
+      </c>
+      <c r="F91" s="3" t="inlineStr">
+        <is>
+          <t>• I like the team that I work with
+• I have learnt a lot of new things
+• I get along really well with my supervisor
+• I have enjoyed doing the work I was employed for
+• Other: Learnt a bit about pneumatic and fuelling logic</t>
+        </is>
+      </c>
+      <c r="G91" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+      <c r="H91" s="3" t="inlineStr">
+        <is>
+          <t>• Helpful / approachable supervisors
+• There is a good team of employees</t>
+        </is>
+      </c>
+      <c r="I91" s="3" t="inlineStr">
+        <is>
+          <t>Supportive and agreeable colleagues and supervisor. Relative freedom while working on new project (R&amp;D type and SBT/depots). PLC Programming, specially structured text Programming. Rare cases of fault findings</t>
+        </is>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>Car park situation (same as last year). Printer too close to the desk. Work planning and prioritization - priorities change multiple times, resulting in mistakes while hopping between tasks; high-priority work is sometimes taken off schedule for months. Lack of clear project specification and expectations at the start of engineering work, and ever-changing specifications. Lack of a clear single stakeholder per project. Untimely project sales handover. Crowded, noisy office space with no dedicated meeting room. Part suppliers' restrictions. Unclear time gap between design and manufacturing. Widespread mindset that Engineering is always responsible for issues. Forced shut-downs using about 40% of paid annual leave without consultation. Not being included in some email chains/discussions but expected to know everything</t>
+        </is>
+      </c>
+      <c r="K91" s="3" t="inlineStr">
+        <is>
+          <t>A clear understanding of the financial aspects of projects' contracts would support better decision-making during the design phase, especially for non-aviation projects. Investment in employees' training and delivering on past promises. Considering Engineering as a finite resource rather than unlimited overhead. Investment in purpose-built tools (i.e. software)</t>
+        </is>
+      </c>
+      <c r="L91" s="3" t="inlineStr">
+        <is>
+          <t>Dealing with other departments. Company having different standards and expectations for different individuals</t>
+        </is>
+      </c>
+      <c r="M91" s="3" t="inlineStr">
+        <is>
+          <t>• This is my chosen career path
+• I enjoy working in this role
+• I want to stay in this area of work
+• This role fulfils my needs and expectations
+• Other: I enjoy the role, but to be honest, I'm not sure about my future</t>
+        </is>
+      </c>
+      <c r="N91" s="3" t="inlineStr">
+        <is>
+          <t>Going over new designs, control logics, and R&amp;D type projects, investigating new products/standards, and trying to analyse systems and/or fault find. Also enjoyed programming while setting up the CAN interface on Volvo FMs</t>
+        </is>
+      </c>
+      <c r="O91" s="3" t="inlineStr">
+        <is>
+          <t>Copy &amp; pasting with minor changes and having to do unnecessary reworks due to last-minute spec changes</t>
+        </is>
+      </c>
+      <c r="P91" s="3" t="inlineStr">
+        <is>
+          <t>Engineering team; supplied separately as a typed docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="96" customHeight="1">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Ehsan Barani</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Confirmed by elimination — the register entry Barani, Ehsan is the only name from the requested engineering list not otherwise accounted for in this document, matching this unnamed section</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Engineering docx, unnamed section between Behzad Moazeni and Liam McNamara</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>Not extractable (older form-field format)</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>I enjoy working in a challenging environment that encourages continuous learning and professional growth. Since joining the company, I have gained valuable new skills and experience through solving complex technical problems. I also appreciate the supportive engineering team, where colleagues are willing to share knowledge and help one another. I enjoy the work I was employed to do and see opportunities to continue developing my career with the company</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>Car park</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>Providing additional training opportunities and dedicated time for professional development in key technical areas would help employees continue building their skills and knowledge. Improving the availability of parking spaces for the engineering team would also enhance convenience and the overall workplace experience</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="inlineStr">
+        <is>
+          <t>I find it most challenging when working on new and unfamiliar tasks under tight deadlines. Balancing rapid learning with delivering accurate, high-quality work can be demanding, but I enjoy the challenge and the opportunity to grow</t>
+        </is>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>I am most interested in the variety of engineering work and the opportunity to continuously learn new skills. I have particularly enjoyed gaining experience in hydraulic and pneumatic systems, which were new areas for me</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>There are no significant aspects of my role that I find least interesting, as each task offers valuable learning opportunities</t>
+        </is>
+      </c>
+      <c r="P92" s="2" t="inlineStr">
+        <is>
+          <t>Name not given on this form; identified by elimination as the remaining name on the engineering list (Ehsan Barani), positioned between Behzad Moazeni and Liam McNamara in the document. This section's tick-boxes use an older Word form-field format that could not be read reliably, so Q1/Q1.1/Q2/Q5 are left blank rather than guessed; the written answers are transcribed in full.</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="96" customHeight="1">
+      <c r="A93" s="3" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>Liam McNamara</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed — exact match (register: McNamara, Liam)</t>
+        </is>
+      </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Engineering docx, Liam McNamara section</t>
+        </is>
+      </c>
+      <c r="F93" s="3" t="inlineStr">
+        <is>
+          <t>• I like the team that I work with
+• I have learnt a lot of new things
+• The job is what I expected it to be
+• I get along really well with my supervisor
+• I have enjoyed doing the work I was employed for
+• I see myself developing further with this company</t>
+        </is>
+      </c>
+      <c r="G93" s="3" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="H93" s="3" t="inlineStr">
+        <is>
+          <t>• Good culture within organisation
+• Helpful / approachable supervisors
+• Recommend this company to others
+• There is a good team of employees
+• Practices to encourage social / employee involvement</t>
+        </is>
+      </c>
       <c r="I93" s="3" t="inlineStr">
         <is>
-          <t>I enjoy writing manuals for many different trucks that have unique features. I like the flexibility in the work hours, where you can make up hours later in the week or extra hours at night or on the weekend</t>
+          <t>Good team, good company culture. Reasonable expectations regarding initial domain specific knowledge</t>
         </is>
       </c>
       <c r="J93" s="3" t="inlineStr">
         <is>
-          <t>Dislike the fork lift traffic</t>
+          <t>Pressuring other departments with a visibly heavier workload than my own to finish jobs</t>
         </is>
       </c>
       <c r="K93" s="3" t="inlineStr">
         <is>
-          <t>More rooms / partitions within the office to cut down on background noise, ensuring the HVAC system is working optimally</t>
+          <t>Improve time sheet / job logging system. Separate break and meeting rooms. More parking</t>
         </is>
       </c>
       <c r="L93" s="3" t="inlineStr">
         <is>
-          <t>Making sure I do my allocated hours even if I get my work done before the minimum hour threshold. Completing all the user manuals on time before the trucks leave the site</t>
+          <t>Coordinating warranty with other departments. Settling large sets of fleetwide warranty claims</t>
         </is>
       </c>
       <c r="M93" s="3" t="inlineStr">
         <is>
           <t>• I enjoy working in this role
-• I want to stay in this area of work</t>
+• This role fulfils my needs and expectations</t>
         </is>
       </c>
       <c r="N93" s="3" t="inlineStr">
         <is>
-          <t>Writing new manuals and improving the explanation of how all the systems operate</t>
+          <t>Trialling new design features and R&amp;D work, such as the 360 degree camera setup</t>
         </is>
       </c>
       <c r="O93" s="3" t="inlineStr">
         <is>
-          <t>Printing lots of pages - I don't like over using the printer and worry if there is enough ink to print the work</t>
+          <t>Troubleshooting web development issues on the ATG portal</t>
         </is>
       </c>
       <c r="P93" s="3" t="inlineStr">
         <is>
-          <t>'This is my chosen career path' left unticked, but annotated alongside: 'More looking into an engineering position' - suggests interest in moving into an engineering role</t>
+          <t>Engineering team; supplied separately as a typed docx</t>
         </is>
       </c>
     </row>
@@ -9222,17 +9224,17 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Mitchell Frick</t>
+          <t>Luke Moran</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Confirmed — exact match (register: Frick, Mitchell)</t>
+          <t>Confirmed — exact match (register: Moran, Luke)</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Engineering docx, Mitchell Frick section</t>
+          <t>Engineering docx, Luke Moran section</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -9240,7 +9242,6 @@
           <t>• I like the team that I work with
 • I have learnt a lot of new things
 • The job is what I expected it to be
-• This job is harder than I expected
 • I get along really well with my supervisor
 • I have enjoyed doing the work I was employed for
 • I see myself developing further with this company</t>
@@ -9248,7 +9249,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -9265,72 +9266,166 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
+          <t>I enjoy writing manuals for many different trucks that have unique features. I like the flexibility in the work hours, where you can make up hours later in the week or extra hours at night or on the weekend</t>
+        </is>
+      </c>
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>Dislike the fork lift traffic</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr">
+        <is>
+          <t>More rooms / partitions within the office to cut down on background noise, ensuring the HVAC system is working optimally</t>
+        </is>
+      </c>
+      <c r="L94" s="2" t="inlineStr">
+        <is>
+          <t>Making sure I do my allocated hours even if I get my work done before the minimum hour threshold. Completing all the user manuals on time before the trucks leave the site</t>
+        </is>
+      </c>
+      <c r="M94" s="2" t="inlineStr">
+        <is>
+          <t>• I enjoy working in this role
+• I want to stay in this area of work</t>
+        </is>
+      </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>Writing new manuals and improving the explanation of how all the systems operate</t>
+        </is>
+      </c>
+      <c r="O94" s="2" t="inlineStr">
+        <is>
+          <t>Printing lots of pages - I don't like over using the printer and worry if there is enough ink to print the work</t>
+        </is>
+      </c>
+      <c r="P94" s="2" t="inlineStr">
+        <is>
+          <t>'This is my chosen career path' left unticked, but annotated alongside: 'More looking into an engineering position' - suggests interest in moving into an engineering role</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="96" customHeight="1">
+      <c r="A95" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="3" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>Mitchell Frick</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed — exact match (register: Frick, Mitchell)</t>
+        </is>
+      </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Engineering docx, Mitchell Frick section</t>
+        </is>
+      </c>
+      <c r="F95" s="3" t="inlineStr">
+        <is>
+          <t>• I like the team that I work with
+• I have learnt a lot of new things
+• The job is what I expected it to be
+• This job is harder than I expected
+• I get along really well with my supervisor
+• I have enjoyed doing the work I was employed for
+• I see myself developing further with this company</t>
+        </is>
+      </c>
+      <c r="G95" s="3" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+      <c r="H95" s="3" t="inlineStr">
+        <is>
+          <t>• Good communication within organisation
+• Helpful / approachable supervisors
+• Career development opportunities
+• There is a good team of employees
+• Good culture within organisation
+• There is opportunity to grow within the company
+• Recommend this company to others
+• Practices to encourage social / employee involvement</t>
+        </is>
+      </c>
+      <c r="I95" s="3" t="inlineStr">
+        <is>
           <t>I enjoy the type of work that is done and the proximity of the workshop and the office allowing for quick feedback between production and workshop teams. Having more design reviews with sales/leadership has been helpful to ensure that we're getting the designs right</t>
         </is>
       </c>
-      <c r="J94" s="2" t="inlineStr">
+      <c r="J95" s="3" t="inlineStr">
         <is>
           <t>Engineering is the first to blame on most of the occasions if something goes wrong, unless it can be proved to be otherwise</t>
         </is>
       </c>
-      <c r="K94" s="2" t="inlineStr">
+      <c r="K95" s="3" t="inlineStr">
         <is>
           <t>Getting more opportunities for feedback/reviews within engineering. Finding some way to relieve the pressure of consecutive high priority tasks</t>
         </is>
       </c>
-      <c r="L94" s="2" t="inlineStr">
+      <c r="L95" s="3" t="inlineStr">
         <is>
           <t>Frequently jumping from task to task. Having to maintain support for multiple projects whilst also working on new designs. Not having enough time to do thorough reviews of designs with the team</t>
         </is>
       </c>
-      <c r="M94" s="2" t="inlineStr">
+      <c r="M95" s="3" t="inlineStr">
         <is>
           <t>• This is my chosen career path
 • I enjoy working in this role
 • I want to stay in this area of work</t>
         </is>
       </c>
-      <c r="N94" s="2" t="inlineStr">
+      <c r="N95" s="3" t="inlineStr">
         <is>
           <t>Circuit design. Standards review</t>
         </is>
       </c>
-      <c r="O94" s="2" t="inlineStr">
+      <c r="O95" s="3" t="inlineStr">
         <is>
           <t>BOM generation. 3D modelling</t>
         </is>
       </c>
-      <c r="P94" s="2" t="inlineStr">
+      <c r="P95" s="3" t="inlineStr">
         <is>
           <t>Annotated 'Competing priorities - design timeframe - workshop assistance' against 'harder than I expected'; annotated 'Work life balance - extra working hours to keep up with deadlines, reduces efficiency' against Q1.1; annotated '(Work life balance)' against 'This role fulfils my needs and expectations' (left unticked)</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="96" customHeight="1">
-      <c r="A95" s="3" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
+    <row r="96" ht="96" customHeight="1">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C95" s="3" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Sai Vivek Yedlapati</t>
         </is>
       </c>
-      <c r="D95" s="3" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>Confirmed — exact match (register: Yedlapati, Sai Vivek)</t>
         </is>
       </c>
-      <c r="E95" s="3" t="inlineStr">
+      <c r="E96" s="2" t="inlineStr">
         <is>
           <t>Engineering docx, Sai Vivek Yedlapati section</t>
         </is>
       </c>
-      <c r="F95" s="3" t="inlineStr">
+      <c r="F96" s="2" t="inlineStr">
         <is>
           <t>• I like the team that I work with
 • I have learnt a lot of new things
@@ -9339,12 +9434,12 @@
 • I see myself developing further with this company</t>
         </is>
       </c>
-      <c r="G95" s="3" t="inlineStr">
+      <c r="G96" s="2" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="H95" s="3" t="inlineStr">
+      <c r="H96" s="2" t="inlineStr">
         <is>
           <t>• Helpful / approachable supervisors
 • Career development opportunities
@@ -9352,27 +9447,27 @@
 • There is opportunity to grow within the company</t>
         </is>
       </c>
-      <c r="I95" s="3" t="inlineStr">
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>Challenging and interesting work. Great team and good people to work with. Supportive work environment. Opportunities to travel for work</t>
         </is>
       </c>
-      <c r="J95" s="3" t="inlineStr">
+      <c r="J96" s="2" t="inlineStr">
         <is>
           <t>Justification and normalisation of overtime; no clear definition of 'reasonable OT'. Review process not designed for the Engineering Team, KPIs not robust or aligned with expected performance. Unclear project ownership and accountability - too many people provide input but decision-making responsibility is unclear. Some procedures place excessive demands on the engineering team. Insufficient time allocated for R&amp;D and testing. Wants greater flexibility around mandatory annual leave, particularly December. Limited parking availability and blocked parking spaces</t>
         </is>
       </c>
-      <c r="K95" s="3" t="inlineStr">
+      <c r="K96" s="2" t="inlineStr">
         <is>
           <t>Implement Agile working practices to improve project planning, communication and delivery. Increase focus on design quality through structured internal engineering reviews. Adopt more capable engineering design software (e.g. EPLAN). Modernise approval processes through digital workflows (warranty approvals, leave requests currently manual). Clearer role definitions so management doesn't struggle with people volunteering for work</t>
         </is>
       </c>
-      <c r="L95" s="3" t="inlineStr">
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>Lack of technical supervision - no dedicated technical supervisor for structured guidance, limiting learning and growth. Lack of formal on-the-job training programme. Balancing supervisory responsibilities with direct job execution creates workload pressure</t>
         </is>
       </c>
-      <c r="M95" s="3" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
         <is>
           <t>• This is my chosen career path
 • I enjoy working in this role
@@ -9380,99 +9475,19 @@
 • Other: The role is going okay for now, but I need to see growth for long term development (like management level)</t>
         </is>
       </c>
-      <c r="N95" s="3" t="inlineStr">
+      <c r="N96" s="2" t="inlineStr">
         <is>
           <t>Problem solving, strategy, engineering, customer relations, design, managing, software</t>
         </is>
       </c>
-      <c r="O95" s="3" t="inlineStr">
+      <c r="O96" s="2" t="inlineStr">
         <is>
           <t>Solving the same problems over and over again (repetitive tasks). Chasing other departments to get the work done</t>
         </is>
       </c>
-      <c r="P95" s="3" t="inlineStr">
+      <c r="P96" s="2" t="inlineStr">
         <is>
           <t>Also wrote against Q1 Other: 'Warranty responsibility part of the job is not clear as we have a dedicated person for that role' (box not ticked)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="96" customHeight="1">
-      <c r="A96" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>Engineering</t>
-        </is>
-      </c>
-      <c r="C96" s="2" t="inlineStr">
-        <is>
-          <t>Vahid Shirazi</t>
-        </is>
-      </c>
-      <c r="D96" s="2" t="inlineStr">
-        <is>
-          <t>Confirmed — exact match (register: Shirazi, Vahid)</t>
-        </is>
-      </c>
-      <c r="E96" s="2" t="inlineStr">
-        <is>
-          <t>Engineering docx, Vahid Shirazi section</t>
-        </is>
-      </c>
-      <c r="F96" s="2" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="G96" s="2" t="inlineStr">
-        <is>
-          <t>Not extractable (older form-field format)</t>
-        </is>
-      </c>
-      <c r="H96" s="2" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="I96" s="2" t="inlineStr">
-        <is>
-          <t>The engineering environment is excellent, the work is challenging, and there are always opportunities to learn new things</t>
-        </is>
-      </c>
-      <c r="J96" s="2" t="inlineStr">
-        <is>
-          <t>The scheduling is poorly managed, and technicians are prioritised over engineers</t>
-        </is>
-      </c>
-      <c r="K96" s="2" t="inlineStr">
-        <is>
-          <t>I feel the company does not allow sufficient time for engineering work, which prevents us from optimising our designs. The company needs to improve its scheduling - it is common for the company to not allocate adequate time for the design process, which can lead to an increase in mistakes. The company also needs to find a solution for car parking - a significant amount of time is wasted each morning searching for a suitable car park</t>
-        </is>
-      </c>
-      <c r="L96" s="2" t="inlineStr">
-        <is>
-          <t>The company needs to plan and send engineers for training to learn new skills, however this does not happen in practice, yet the company still expects the engineering department to produce designs in specialised areas such as hydraulics. The company needs to improve its scheduling and allocate adequate time to the engineering department for thinking and designing</t>
-        </is>
-      </c>
-      <c r="M96" s="2" t="inlineStr">
-        <is>
-          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
-        </is>
-      </c>
-      <c r="N96" s="2" t="inlineStr">
-        <is>
-          <t>I am interested in this job because of the work challenges and the opportunity to work with structural, hydraulic, and pneumatic design. I also particularly enjoy the engineering department culture</t>
-        </is>
-      </c>
-      <c r="O96" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="P96" s="2" t="inlineStr">
-        <is>
-          <t>This section's tick-boxes use an older Word form-field format that could not be read reliably, so Q1/Q1.1/Q2/Q5 are left blank rather than guessed; the written answers are transcribed in full. No separate 'least' answer was given at Q5.1</t>
         </is>
       </c>
     </row>
@@ -9487,20 +9502,100 @@
       </c>
       <c r="C97" s="3" t="inlineStr">
         <is>
+          <t>Vahid Shirazi</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed — exact match (register: Shirazi, Vahid)</t>
+        </is>
+      </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Engineering docx, Vahid Shirazi section</t>
+        </is>
+      </c>
+      <c r="F97" s="3" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="G97" s="3" t="inlineStr">
+        <is>
+          <t>Not extractable (older form-field format)</t>
+        </is>
+      </c>
+      <c r="H97" s="3" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="I97" s="3" t="inlineStr">
+        <is>
+          <t>The engineering environment is excellent, the work is challenging, and there are always opportunities to learn new things</t>
+        </is>
+      </c>
+      <c r="J97" s="3" t="inlineStr">
+        <is>
+          <t>The scheduling is poorly managed, and technicians are prioritised over engineers</t>
+        </is>
+      </c>
+      <c r="K97" s="3" t="inlineStr">
+        <is>
+          <t>I feel the company does not allow sufficient time for engineering work, which prevents us from optimising our designs. The company needs to improve its scheduling - it is common for the company to not allocate adequate time for the design process, which can lead to an increase in mistakes. The company also needs to find a solution for car parking - a significant amount of time is wasted each morning searching for a suitable car park</t>
+        </is>
+      </c>
+      <c r="L97" s="3" t="inlineStr">
+        <is>
+          <t>The company needs to plan and send engineers for training to learn new skills, however this does not happen in practice, yet the company still expects the engineering department to produce designs in specialised areas such as hydraulics. The company needs to improve its scheduling and allocate adequate time to the engineering department for thinking and designing</t>
+        </is>
+      </c>
+      <c r="M97" s="3" t="inlineStr">
+        <is>
+          <t>• Not extractable — checkboxes in this document use an older Word form-field format that could not be read</t>
+        </is>
+      </c>
+      <c r="N97" s="3" t="inlineStr">
+        <is>
+          <t>I am interested in this job because of the work challenges and the opportunity to work with structural, hydraulic, and pneumatic design. I also particularly enjoy the engineering department culture</t>
+        </is>
+      </c>
+      <c r="O97" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P97" s="3" t="inlineStr">
+        <is>
+          <t>This section's tick-boxes use an older Word form-field format that could not be read reliably, so Q1/Q1.1/Q2/Q5 are left blank rather than guessed; the written answers are transcribed in full. No separate 'least' answer was given at Q5.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="96" customHeight="1">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
           <t>Josh Cho</t>
         </is>
       </c>
-      <c r="D97" s="3" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>Confirmed — Young Wan (Josh) Cho (register: Cho, Young Wan (Josh))</t>
         </is>
       </c>
-      <c r="E97" s="3" t="inlineStr">
+      <c r="E98" s="2" t="inlineStr">
         <is>
           <t>Engineering PDF, Josh Cho (typed, 14 pages)</t>
         </is>
       </c>
-      <c r="F97" s="3" t="inlineStr">
+      <c r="F98" s="2" t="inlineStr">
         <is>
           <t>• I like the team that I work with
 • I have learnt a lot of new things
@@ -9510,12 +9605,12 @@
 • I see myself developing further with this company</t>
         </is>
       </c>
-      <c r="G97" s="3" t="inlineStr">
+      <c r="G98" s="2" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="H97" s="3" t="inlineStr">
+      <c r="H98" s="2" t="inlineStr">
         <is>
           <t>• Good communication within organisation
 • Helpful / approachable supervisors
@@ -9526,27 +9621,27 @@
 • Recommend this company to others</t>
         </is>
       </c>
-      <c r="I97" s="3" t="inlineStr">
+      <c r="I98" s="2" t="inlineStr">
         <is>
           <t>Working with good teammates</t>
         </is>
       </c>
-      <c r="J97" s="3" t="inlineStr">
+      <c r="J98" s="2" t="inlineStr">
         <is>
           <t>Still need to improve team management and work process development</t>
         </is>
       </c>
-      <c r="K97" s="3" t="inlineStr">
+      <c r="K98" s="2" t="inlineStr">
         <is>
           <t>Sometimes tasks are started based on verbal instructions without a formal process, meeting, or clear written direction. In these situations, the work can become less efficient because expectations, priorities, and responsibilities are not always clearly aligned from the beginning. Having clearer communication, more structured planning, and documented instructions where appropriate would help improve efficiency, reduce misunderstandings, and support better teamwork</t>
         </is>
       </c>
-      <c r="L97" s="3" t="inlineStr">
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>Managing parts ordering and clearly defining the order scope before a project starts. Sometimes parts need to be ordered from production or arranged based on limited information, which can make it difficult to confirm exactly what is required. Clearer communication around parts requirements, project scope, and responsibilities would make this part of the job easier to manage</t>
         </is>
       </c>
-      <c r="M97" s="3" t="inlineStr">
+      <c r="M98" s="2" t="inlineStr">
         <is>
           <t>• This is my chosen career path
 • I enjoy working in this role
@@ -9554,47 +9649,47 @@
 • This role fulfils my needs and expectations</t>
         </is>
       </c>
-      <c r="N97" s="3" t="inlineStr">
+      <c r="N98" s="2" t="inlineStr">
         <is>
           <t>Engineering design, problem-solving, and working on practical technical solutions. Learning more about standards, compliance, manufacturing processes, and how design decisions affect the final product</t>
         </is>
       </c>
-      <c r="O97" s="3" t="inlineStr">
+      <c r="O98" s="2" t="inlineStr">
         <is>
           <t>Car park (handwritten addition)</t>
         </is>
       </c>
-      <c r="P97" s="3" t="inlineStr">
+      <c r="P98" s="2" t="inlineStr">
         <is>
           <t>Engineering team; typed form, submitted as PDF</t>
         </is>
       </c>
     </row>
-    <row r="98" ht="96" customHeight="1">
-      <c r="A98" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
+    <row r="99" ht="96" customHeight="1">
+      <c r="A99" s="3" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="3" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C98" s="2" t="inlineStr">
+      <c r="C99" s="3" t="inlineStr">
         <is>
           <t>Muhammad Saad Zia</t>
         </is>
       </c>
-      <c r="D98" s="2" t="inlineStr">
+      <c r="D99" s="3" t="inlineStr">
         <is>
           <t>Confirmed — exact match (register: Zia, Muhammad Saad)</t>
         </is>
       </c>
-      <c r="E98" s="2" t="inlineStr">
+      <c r="E99" s="3" t="inlineStr">
         <is>
           <t>Engineering PDF, Muhammad Saad Zia (13 pages)</t>
         </is>
       </c>
-      <c r="F98" s="2" t="inlineStr">
+      <c r="F99" s="3" t="inlineStr">
         <is>
           <t>• I like the team that I work with
 • I have learnt a lot of new things
@@ -9604,12 +9699,12 @@
 • I see myself developing further with this company</t>
         </is>
       </c>
-      <c r="G98" s="2" t="inlineStr">
+      <c r="G99" s="3" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="H98" s="2" t="inlineStr">
+      <c r="H99" s="3" t="inlineStr">
         <is>
           <t>• Helpful / approachable supervisors
 • Career development opportunities
@@ -9618,27 +9713,27 @@
 • Recommend this company to others (annotated 'have gotten poor')</t>
         </is>
       </c>
-      <c r="I98" s="2" t="inlineStr">
+      <c r="I99" s="3" t="inlineStr">
         <is>
           <t>I genuinely enjoy the technical variety of work. Delivering projects for clients all over the world has been a fantastic growth opportunity. What I would like to see improve is a more structured handover and mentoring time as senior responsibilities transition to me, and more realistic project scoping at the planning stage</t>
         </is>
       </c>
-      <c r="J98" s="2" t="inlineStr">
+      <c r="J99" s="3" t="inlineStr">
         <is>
           <t>See likes column - handover/mentoring structure and project scoping realism</t>
         </is>
       </c>
-      <c r="K98" s="2" t="inlineStr">
+      <c r="K99" s="3" t="inlineStr">
         <is>
           <t>More structured time for knowledge transfer from senior engineers during role transfer and transitions, and earlier engineering input into project timelines at the quoting/scoping stage to ensure deadlines reflect actual scope of work</t>
         </is>
       </c>
-      <c r="L98" s="2" t="inlineStr">
+      <c r="L99" s="3" t="inlineStr">
         <is>
           <t>Building deep first-principles knowledge in pressure vessel design and hydraulics/pneumatics while balancing a high project workload. Actively addressing this through self learning and the AS1210 standard, but more structured access to senior engineering knowledge would accelerate this</t>
         </is>
       </c>
-      <c r="M98" s="2" t="inlineStr">
+      <c r="M99" s="3" t="inlineStr">
         <is>
           <t>• This is my chosen career path
 • I enjoy working in this role
@@ -9646,47 +9741,47 @@
 • This role fulfils my needs and expectations</t>
         </is>
       </c>
-      <c r="N98" s="2" t="inlineStr">
+      <c r="N99" s="3" t="inlineStr">
         <is>
           <t>Ownership of complex projects like the CPC Hydrant. Seeing a design go from concept through to FAT and into the field is genuinely rewarding</t>
         </is>
       </c>
-      <c r="O98" s="2" t="inlineStr">
+      <c r="O99" s="3" t="inlineStr">
         <is>
           <t>Administrative rework caused by compressed deadlines that don't match project scope</t>
         </is>
       </c>
-      <c r="P98" s="2" t="inlineStr">
+      <c r="P99" s="3" t="inlineStr">
         <is>
           <t>Annotated 'Mixed' against Good communication/Good culture (left unticked); annotated 'have gotten poor' next to Recommend this company to others (ticked but qualified)</t>
         </is>
       </c>
     </row>
-    <row r="99" ht="96" customHeight="1">
-      <c r="A99" s="3" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="3" t="inlineStr">
+    <row r="100" ht="96" customHeight="1">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr">
+      <c r="C100" s="2" t="inlineStr">
         <is>
           <t>Patrick Tio</t>
         </is>
       </c>
-      <c r="D99" s="3" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>Register lists 'Patrice Tio' (register: Tio, Patrice) — the form itself is signed and titled 'Patrick Tio' throughout, so this may be a register typo or a preferred name; flagging the discrepancy rather than resolving it either way</t>
         </is>
       </c>
-      <c r="E99" s="3" t="inlineStr">
+      <c r="E100" s="2" t="inlineStr">
         <is>
           <t>Engineering PDF, Patrick Tio (13 pages)</t>
         </is>
       </c>
-      <c r="F99" s="3" t="inlineStr">
+      <c r="F100" s="2" t="inlineStr">
         <is>
           <t>• I like the team that I work with
 • I have learnt a lot of new things
@@ -9695,63 +9790,63 @@
 • I see myself developing further with this company</t>
         </is>
       </c>
-      <c r="G99" s="3" t="inlineStr">
+      <c r="G100" s="2" t="inlineStr">
         <is>
           <t>Good / Satisfactory (both appear marked)</t>
         </is>
       </c>
-      <c r="H99" s="3" t="inlineStr">
+      <c r="H100" s="2" t="inlineStr">
         <is>
           <t>• Good communication within organisation
 • Helpful / approachable supervisors
 • There is a good team of employees</t>
         </is>
       </c>
-      <c r="I99" s="3" t="inlineStr">
+      <c r="I100" s="2" t="inlineStr">
         <is>
           <t>Lots of jobs</t>
         </is>
       </c>
-      <c r="J99" s="3" t="inlineStr">
+      <c r="J100" s="2" t="inlineStr">
         <is>
           <t>Schedule of job, working hours</t>
         </is>
       </c>
-      <c r="K99" s="3" t="inlineStr">
+      <c r="K100" s="2" t="inlineStr">
         <is>
           <t>Better work life balance</t>
         </is>
       </c>
-      <c r="L99" s="3" t="inlineStr">
+      <c r="L100" s="2" t="inlineStr">
         <is>
           <t>Understanding customer request</t>
         </is>
       </c>
-      <c r="M99" s="3" t="inlineStr">
+      <c r="M100" s="2" t="inlineStr">
         <is>
           <t>• This is my chosen career path
 • I enjoy working in this role
 • I want to stay in this area of work</t>
         </is>
       </c>
-      <c r="N99" s="3" t="inlineStr">
+      <c r="N100" s="2" t="inlineStr">
         <is>
           <t>Doing design</t>
         </is>
       </c>
-      <c r="O99" s="3" t="inlineStr">
+      <c r="O100" s="2" t="inlineStr">
         <is>
           <t>Doing paper work</t>
         </is>
       </c>
-      <c r="P99" s="3" t="inlineStr">
+      <c r="P100" s="2" t="inlineStr">
         <is>
           <t>Engineering team; short handwritten answers</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P99"/>
+  <autoFilter ref="A1:P100"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10343,7 +10438,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6">
@@ -10353,7 +10448,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7">
@@ -10363,7 +10458,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8">
@@ -10373,7 +10468,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -10383,7 +10478,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -10393,7 +10488,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11">
@@ -10462,7 +10557,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20">
@@ -10521,7 +10616,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="28">
@@ -10531,7 +10626,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="29">
@@ -10541,7 +10636,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30">
@@ -10551,7 +10646,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31">
@@ -10561,7 +10656,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="32">
@@ -10571,7 +10666,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="33">
@@ -10581,7 +10676,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="34">
@@ -10591,7 +10686,7 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="35">
@@ -10630,7 +10725,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="41">
@@ -10640,7 +10735,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="42">
@@ -10650,7 +10745,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43">
@@ -10660,7 +10755,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44">
@@ -10733,7 +10828,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Employee Feedback 2026 — summary of all 98 responses</t>
+          <t>Employee Feedback 2026 — summary of all 99 responses</t>
         </is>
       </c>
     </row>
@@ -10775,7 +10870,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Source</t>
@@ -10783,7 +10878,7 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>Three scanned bundles (Employee Feedback forms 1, 2 and 3 — 40, 94 and 68 pages) covering the 87 workshop/office respondents, plus 11 engineering team reviews supplied separately: eight as sections of one Word document and three as individually typed PDFs (Josh Cho, Muhammad Saad Zia, Patrick Tio). Every page was read individually.</t>
+          <t>Three scanned bundles (Employee Feedback forms 1, 2 and 3 — 40, 94 and 68 pages) covering most of the 88 workshop/office respondents, plus 11 engineering team reviews supplied separately: eight as sections of one Word document and three as individually typed PDFs (Josh Cho, Muhammad Saad Zia, Patrick Tio). One further workshop/office form (Rita Kelly) arrived as a single standalone scanned page with no cover or signature; her name was confirmed by Geoff and matched to the personnel register. Every page was read individually.</t>
         </is>
       </c>
     </row>
@@ -10795,7 +10890,7 @@
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>98 completed feedback forms are recorded, one row each, on the 'Feedback Responses' tab — 87 workshop/office plus 11 engineering, distinguished by the Team column.</t>
+          <t>99 completed feedback forms are recorded, one row each, on the 'Feedback Responses' tab — 88 workshop/office plus 11 engineering, distinguished by the Team column.</t>
         </is>
       </c>
     </row>

</xml_diff>